<commit_message>
feat: add application tracking (suivi_candidatures.xlsx)
New feature: after each email is sent, the application is automatically
logged to data/suivi_candidatures.xlsx for follow-up tracking.

Files:
- scripts/tracking/tracker.js: appendRow(), getStats(), ensureFile()
- tests/tracker.test.js: 15 tests covering all tracker functions
- prompts/10_start_campaign.txt: added tracking step (step 10)
- prompts/20_deep_research.txt: added tracking step in Phase 2
- package.json: added tracking and tracking:stats scripts

Tracking columns:
- Entreprise, Poste, Lien Offre, Recruteur (email)
- Date DM envoye (auto-filled with current date)
- Lien Entreprise, Notes

Features:
- Auto-creates Excel file if it doesn't exist
- Duplicate detection (same company + position + date)
- Follow-up date calculated (J+7)
- Hyperlinks for URLs
- Frozen header row with blue styling

Tests: 163 passing (was 148)
</commit_message>
<xml_diff>
--- a/data/research/deep_research_results.xlsx
+++ b/data/research/deep_research_results.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="413" uniqueCount="126">
   <si>
     <t>N°</t>
   </si>
@@ -68,97 +68,295 @@
     <t>Raisons du match</t>
   </si>
   <si>
+    <t>Competences manquantes</t>
+  </si>
+  <si>
     <t>Commentaires</t>
   </si>
   <si>
     <t>Statut candidature</t>
   </si>
   <si>
-    <t>TechCorp</t>
-  </si>
-  <si>
-    <t>Backend PHP Developer</t>
-  </si>
-  <si>
-    <t>Casablanca</t>
-  </si>
-  <si>
-    <t>CDI</t>
+    <t>Quik Hire Staffing</t>
+  </si>
+  <si>
+    <t>Frontend Web Developer - HTML, CSS (Remote)</t>
+  </si>
+  <si>
+    <t>Remote (Europe, Middle East &amp; Africa)</t>
   </si>
   <si>
     <t/>
   </si>
   <si>
-    <t>PHP, Laravel, MySQL, Docker</t>
-  </si>
-  <si>
-    <t>LinkedIn</t>
+    <t>https://www.linkedin.com/jobs/view/4456473106</t>
+  </si>
+  <si>
+    <t>linkedin</t>
   </si>
   <si>
     <t>LINKEDIN</t>
   </si>
   <si>
-    <t>18/08/2026</t>
+    <t>20/08/2026</t>
   </si>
   <si>
     <t>UNKNOWN</t>
   </si>
   <si>
-    <t>Tres bon</t>
-  </si>
-  <si>
-    <t>Certaines competences correspondantes; Stack technique tres compatible; Localisation ideale; Technologies matching: PHP, Laravel, MySQL</t>
+    <t>Moyen</t>
+  </si>
+  <si>
+    <t>Peu de competences correspondantes; Stack technique partiellement compatible; Localisation ideale</t>
   </si>
   <si>
     <t>A ENVOYER</t>
   </si>
   <si>
-    <t>WebInc</t>
-  </si>
-  <si>
-    <t>Laravel Developer</t>
-  </si>
-  <si>
-    <t>Rabat</t>
-  </si>
-  <si>
-    <t>PHP, Laravel, Vue.js</t>
-  </si>
-  <si>
-    <t>hr@webinc.com</t>
-  </si>
-  <si>
-    <t>Indeed</t>
-  </si>
-  <si>
-    <t>EMAIL</t>
-  </si>
-  <si>
-    <t>Moyen</t>
-  </si>
-  <si>
-    <t>Peu de competences correspondantes; Stack technique tres compatible; Localisation eloignee; Technologies matching: PHP, Laravel, Vue.js</t>
-  </si>
-  <si>
-    <t>StartupX</t>
-  </si>
-  <si>
-    <t>Frontend React Developer</t>
-  </si>
-  <si>
-    <t>Remote</t>
-  </si>
-  <si>
-    <t>Freelance</t>
-  </si>
-  <si>
-    <t>React, TypeScript, Node.js</t>
+    <t>SQLI</t>
+  </si>
+  <si>
+    <t>Développeur Full Stack Node JS/Vue JS</t>
+  </si>
+  <si>
+    <t>Oujda, Maroc (À distance)</t>
+  </si>
+  <si>
+    <t>Vue.js, Node.js</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/jobs/view/4341041659</t>
+  </si>
+  <si>
+    <t>Peu de competences correspondantes; Stack technique partiellement compatible; Localisation eloignee; Technologies matching: Vue.js; Localisation: Oujda, Maroc (À distance) (vous cherchez: Casablanca)</t>
+  </si>
+  <si>
+    <t>Node.js</t>
+  </si>
+  <si>
+    <t>Conquer AI</t>
+  </si>
+  <si>
+    <t>Software Engineer</t>
+  </si>
+  <si>
+    <t>Remote (North Africa)</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/jobs/view/4453889271</t>
+  </si>
+  <si>
+    <t>Kazacube</t>
+  </si>
+  <si>
+    <t>Développeur senior</t>
+  </si>
+  <si>
+    <t>Casablanca, Maroc (Hybride)</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/jobs/view/4454028605</t>
   </si>
   <si>
     <t>Faible</t>
   </si>
   <si>
-    <t>Peu de competences correspondantes; Localisation ideale; Technologies matching: React, TypeScript</t>
+    <t>Saham Bank</t>
+  </si>
+  <si>
+    <t>Développeur (H/F)</t>
+  </si>
+  <si>
+    <t>Casablanca, Maroc (Sur site)</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/jobs/view/4453416435</t>
+  </si>
+  <si>
+    <t>Sofrecom Maroc</t>
+  </si>
+  <si>
+    <t>Data Engineer (F/H)</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/jobs/view/4455274187</t>
+  </si>
+  <si>
+    <t>micro1</t>
+  </si>
+  <si>
+    <t>Full Stack Engineer</t>
+  </si>
+  <si>
+    <t>Remote (Middle East &amp; North Africa)</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/jobs/view/4456307945</t>
+  </si>
+  <si>
+    <t>Software Engineer - Backend (Remote)</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/jobs/view/4456459287</t>
+  </si>
+  <si>
+    <t>Software Engineer, Internal Platforms</t>
+  </si>
+  <si>
+    <t>TypeScript, React, Node.js, PostgreSQL, AWS</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/jobs/view/4455596295</t>
+  </si>
+  <si>
+    <t>Peu de competences correspondantes; Localisation ideale; Technologies matching: TypeScript, React, PostgreSQL</t>
+  </si>
+  <si>
+    <t>TotalEnergies</t>
+  </si>
+  <si>
+    <t>Développeur IT</t>
+  </si>
+  <si>
+    <t>Maroc (Sur site)</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/jobs/view/4445712167</t>
+  </si>
+  <si>
+    <t>Peu de competences correspondantes; Stack technique partiellement compatible; Localisation eloignee; Localisation: Maroc (Sur site) (vous cherchez: Casablanca)</t>
+  </si>
+  <si>
+    <t>DXC Technology Morocco</t>
+  </si>
+  <si>
+    <t>Data Engineer</t>
+  </si>
+  <si>
+    <t>Rabat, Maroc (Hybride)</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/jobs/view/4455771114</t>
+  </si>
+  <si>
+    <t>Peu de competences correspondantes; Stack technique partiellement compatible; Localisation eloignee; Localisation: Rabat, Maroc (Hybride) (vous cherchez: Casablanca)</t>
+  </si>
+  <si>
+    <t>Devoteam</t>
+  </si>
+  <si>
+    <t>Développeur Senior .NET</t>
+  </si>
+  <si>
+    <t>Skhirate, Maroc (Sur site)</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/jobs/view/4318729105</t>
+  </si>
+  <si>
+    <t>Peu de competences correspondantes; Stack technique partiellement compatible; Localisation eloignee; Localisation: Skhirate, Maroc (Sur site) (vous cherchez: Casablanca)</t>
+  </si>
+  <si>
+    <t>Hire Feed</t>
+  </si>
+  <si>
+    <t>JavaScript Frontend Developer (Remote)</t>
+  </si>
+  <si>
+    <t>JavaScript, Java</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/jobs/view/4456446989</t>
+  </si>
+  <si>
+    <t>Peu de competences correspondantes; Localisation ideale; Technologies matching: JavaScript, Java</t>
+  </si>
+  <si>
+    <t>ICD Fullstack ReactJs/NodeJs (Rabat/Casablanca)</t>
+  </si>
+  <si>
+    <t>Rabat, Maroc (Sur site)</t>
+  </si>
+  <si>
+    <t>React, NodeJs</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/jobs/view/4314993223</t>
+  </si>
+  <si>
+    <t>Peu de competences correspondantes; Localisation eloignee; Technologies matching: React; Localisation: Rabat, Maroc (Sur site) (vous cherchez: Casablanca)</t>
+  </si>
+  <si>
+    <t>NodeJs</t>
+  </si>
+  <si>
+    <t>Inetum</t>
+  </si>
+  <si>
+    <t>Fullstack Java/Angular - Sénior</t>
+  </si>
+  <si>
+    <t>Angular, Java</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/jobs/view/4399408720</t>
+  </si>
+  <si>
+    <t>Peu de competences correspondantes; Localisation ideale; Technologies matching: Java</t>
+  </si>
+  <si>
+    <t>Angular</t>
+  </si>
+  <si>
+    <t>Viveris</t>
+  </si>
+  <si>
+    <t>Développeur .Net/Angular Freelance H/F</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/jobs/view/4455368503</t>
+  </si>
+  <si>
+    <t>Peu de competences correspondantes; Localisation ideale</t>
+  </si>
+  <si>
+    <t>Développeur Python</t>
+  </si>
+  <si>
+    <t>Python</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/jobs/view/4437851188</t>
+  </si>
+  <si>
+    <t>Confidential</t>
+  </si>
+  <si>
+    <t>Back End Developer</t>
+  </si>
+  <si>
+    <t>go</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/jobs/view/4453731079</t>
+  </si>
+  <si>
+    <t>Développeur Front End Angular (Rabat/Casablanca)</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/jobs/view/4387864005</t>
+  </si>
+  <si>
+    <t>Peu de competences correspondantes; Localisation eloignee; Localisation: Rabat, Maroc (Hybride) (vous cherchez: Casablanca)</t>
+  </si>
+  <si>
+    <t>Hired</t>
+  </si>
+  <si>
+    <t>Python Engineer (Remote)</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/jobs/view/4456451813</t>
   </si>
   <si>
     <t>Metrique</t>
@@ -198,7 +396,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -211,8 +409,12 @@
       <color rgb="FFFFFFFF"/>
       <sz val="11"/>
     </font>
+    <font>
+      <u/>
+      <color rgb="FF0563C1"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -222,11 +424,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF2E75B6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF00B0F0"/>
       </patternFill>
     </fill>
     <fill>
@@ -257,9 +454,9 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -599,7 +796,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:T4"/>
+  <dimension ref="A1:U21"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -617,11 +814,11 @@
     <col min="16" max="16" width="12" customWidth="1"/>
     <col min="17" max="17" width="18" customWidth="1"/>
     <col min="18" max="18" width="45" customWidth="1"/>
-    <col min="19" max="19" width="30" customWidth="1"/>
-    <col min="20" max="20" width="18" customWidth="1"/>
+    <col min="19" max="20" width="30" customWidth="1"/>
+    <col min="21" max="21" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="25" customHeight="1" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="25" customHeight="1" spans="1:21" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -682,37 +879,40 @@
       <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="U1" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F2" t="s">
         <v>24</v>
       </c>
       <c r="G2" t="s">
+        <v>24</v>
+      </c>
+      <c r="H2" t="s">
+        <v>24</v>
+      </c>
+      <c r="I2" t="s">
+        <v>24</v>
+      </c>
+      <c r="J2" s="2" t="s">
         <v>25</v>
-      </c>
-      <c r="H2" t="s">
-        <v>24</v>
-      </c>
-      <c r="I2" t="s">
-        <v>24</v>
-      </c>
-      <c r="J2" t="s">
-        <v>24</v>
       </c>
       <c r="K2" t="s">
         <v>24</v>
@@ -729,10 +929,10 @@
       <c r="O2" t="s">
         <v>29</v>
       </c>
-      <c r="P2" s="2">
-        <v>80</v>
-      </c>
-      <c r="Q2" s="2" t="s">
+      <c r="P2" s="3">
+        <v>54</v>
+      </c>
+      <c r="Q2" s="3" t="s">
         <v>30</v>
       </c>
       <c r="R2" t="s">
@@ -742,10 +942,13 @@
         <v>24</v>
       </c>
       <c r="T2" t="s">
+        <v>24</v>
+      </c>
+      <c r="U2" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -759,7 +962,7 @@
         <v>35</v>
       </c>
       <c r="E3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F3" t="s">
         <v>24</v>
@@ -771,19 +974,19 @@
         <v>24</v>
       </c>
       <c r="I3" t="s">
+        <v>24</v>
+      </c>
+      <c r="J3" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="J3" t="s">
-        <v>24</v>
-      </c>
       <c r="K3" t="s">
         <v>24</v>
       </c>
       <c r="L3" t="s">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="M3" t="s">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="N3" t="s">
         <v>28</v>
@@ -792,51 +995,54 @@
         <v>29</v>
       </c>
       <c r="P3" s="3">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="Q3" s="3" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="R3" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="S3" t="s">
-        <v>24</v>
+        <v>39</v>
       </c>
       <c r="T3" t="s">
+        <v>24</v>
+      </c>
+      <c r="U3" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C4" t="s">
+        <v>41</v>
+      </c>
+      <c r="D4" t="s">
         <v>42</v>
       </c>
-      <c r="C4" t="s">
+      <c r="E4" t="s">
+        <v>24</v>
+      </c>
+      <c r="F4" t="s">
+        <v>24</v>
+      </c>
+      <c r="G4" t="s">
+        <v>24</v>
+      </c>
+      <c r="H4" t="s">
+        <v>24</v>
+      </c>
+      <c r="I4" t="s">
+        <v>24</v>
+      </c>
+      <c r="J4" s="2" t="s">
         <v>43</v>
-      </c>
-      <c r="D4" t="s">
-        <v>44</v>
-      </c>
-      <c r="E4" t="s">
-        <v>45</v>
-      </c>
-      <c r="F4" t="s">
-        <v>24</v>
-      </c>
-      <c r="G4" t="s">
-        <v>46</v>
-      </c>
-      <c r="H4" t="s">
-        <v>24</v>
-      </c>
-      <c r="I4" t="s">
-        <v>24</v>
-      </c>
-      <c r="J4" t="s">
-        <v>24</v>
       </c>
       <c r="K4" t="s">
         <v>24</v>
@@ -853,24 +1059,1162 @@
       <c r="O4" t="s">
         <v>29</v>
       </c>
-      <c r="P4" s="4">
-        <v>35</v>
-      </c>
-      <c r="Q4" s="4" t="s">
+      <c r="P4" s="3">
+        <v>50</v>
+      </c>
+      <c r="Q4" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="R4" t="s">
+        <v>31</v>
+      </c>
+      <c r="S4" t="s">
+        <v>24</v>
+      </c>
+      <c r="T4" t="s">
+        <v>24</v>
+      </c>
+      <c r="U4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>44</v>
+      </c>
+      <c r="C5" t="s">
+        <v>45</v>
+      </c>
+      <c r="D5" t="s">
+        <v>46</v>
+      </c>
+      <c r="E5" t="s">
+        <v>24</v>
+      </c>
+      <c r="F5" t="s">
+        <v>24</v>
+      </c>
+      <c r="G5" t="s">
+        <v>24</v>
+      </c>
+      <c r="H5" t="s">
+        <v>24</v>
+      </c>
+      <c r="I5" t="s">
+        <v>24</v>
+      </c>
+      <c r="J5" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="R4" t="s">
+      <c r="K5" t="s">
+        <v>24</v>
+      </c>
+      <c r="L5" t="s">
+        <v>26</v>
+      </c>
+      <c r="M5" t="s">
+        <v>27</v>
+      </c>
+      <c r="N5" t="s">
+        <v>28</v>
+      </c>
+      <c r="O5" t="s">
+        <v>29</v>
+      </c>
+      <c r="P5" s="4">
         <v>48</v>
       </c>
-      <c r="S4" t="s">
-        <v>24</v>
-      </c>
-      <c r="T4" t="s">
+      <c r="Q5" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="R5" t="s">
+        <v>31</v>
+      </c>
+      <c r="S5" t="s">
+        <v>24</v>
+      </c>
+      <c r="T5" t="s">
+        <v>24</v>
+      </c>
+      <c r="U5" t="s">
         <v>32</v>
       </c>
     </row>
+    <row r="6" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>49</v>
+      </c>
+      <c r="C6" t="s">
+        <v>50</v>
+      </c>
+      <c r="D6" t="s">
+        <v>51</v>
+      </c>
+      <c r="E6" t="s">
+        <v>24</v>
+      </c>
+      <c r="F6" t="s">
+        <v>24</v>
+      </c>
+      <c r="G6" t="s">
+        <v>24</v>
+      </c>
+      <c r="H6" t="s">
+        <v>24</v>
+      </c>
+      <c r="I6" t="s">
+        <v>24</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="K6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L6" t="s">
+        <v>26</v>
+      </c>
+      <c r="M6" t="s">
+        <v>27</v>
+      </c>
+      <c r="N6" t="s">
+        <v>28</v>
+      </c>
+      <c r="O6" t="s">
+        <v>29</v>
+      </c>
+      <c r="P6" s="4">
+        <v>48</v>
+      </c>
+      <c r="Q6" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="R6" t="s">
+        <v>31</v>
+      </c>
+      <c r="S6" t="s">
+        <v>24</v>
+      </c>
+      <c r="T6" t="s">
+        <v>24</v>
+      </c>
+      <c r="U6" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="7" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>53</v>
+      </c>
+      <c r="C7" t="s">
+        <v>54</v>
+      </c>
+      <c r="D7" t="s">
+        <v>51</v>
+      </c>
+      <c r="E7" t="s">
+        <v>24</v>
+      </c>
+      <c r="F7" t="s">
+        <v>24</v>
+      </c>
+      <c r="G7" t="s">
+        <v>24</v>
+      </c>
+      <c r="H7" t="s">
+        <v>24</v>
+      </c>
+      <c r="I7" t="s">
+        <v>24</v>
+      </c>
+      <c r="J7" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="K7" t="s">
+        <v>24</v>
+      </c>
+      <c r="L7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N7" t="s">
+        <v>28</v>
+      </c>
+      <c r="O7" t="s">
+        <v>29</v>
+      </c>
+      <c r="P7" s="4">
+        <v>48</v>
+      </c>
+      <c r="Q7" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="R7" t="s">
+        <v>31</v>
+      </c>
+      <c r="S7" t="s">
+        <v>24</v>
+      </c>
+      <c r="T7" t="s">
+        <v>24</v>
+      </c>
+      <c r="U7" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>56</v>
+      </c>
+      <c r="C8" t="s">
+        <v>57</v>
+      </c>
+      <c r="D8" t="s">
+        <v>58</v>
+      </c>
+      <c r="E8" t="s">
+        <v>24</v>
+      </c>
+      <c r="F8" t="s">
+        <v>24</v>
+      </c>
+      <c r="G8" t="s">
+        <v>24</v>
+      </c>
+      <c r="H8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I8" t="s">
+        <v>24</v>
+      </c>
+      <c r="J8" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="K8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L8" t="s">
+        <v>26</v>
+      </c>
+      <c r="M8" t="s">
+        <v>27</v>
+      </c>
+      <c r="N8" t="s">
+        <v>28</v>
+      </c>
+      <c r="O8" t="s">
+        <v>29</v>
+      </c>
+      <c r="P8" s="4">
+        <v>47</v>
+      </c>
+      <c r="Q8" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="R8" t="s">
+        <v>31</v>
+      </c>
+      <c r="S8" t="s">
+        <v>24</v>
+      </c>
+      <c r="T8" t="s">
+        <v>24</v>
+      </c>
+      <c r="U8" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="9" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>21</v>
+      </c>
+      <c r="C9" t="s">
+        <v>60</v>
+      </c>
+      <c r="D9" t="s">
+        <v>23</v>
+      </c>
+      <c r="E9" t="s">
+        <v>24</v>
+      </c>
+      <c r="F9" t="s">
+        <v>24</v>
+      </c>
+      <c r="G9" t="s">
+        <v>24</v>
+      </c>
+      <c r="H9" t="s">
+        <v>24</v>
+      </c>
+      <c r="I9" t="s">
+        <v>24</v>
+      </c>
+      <c r="J9" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="K9" t="s">
+        <v>24</v>
+      </c>
+      <c r="L9" t="s">
+        <v>26</v>
+      </c>
+      <c r="M9" t="s">
+        <v>27</v>
+      </c>
+      <c r="N9" t="s">
+        <v>28</v>
+      </c>
+      <c r="O9" t="s">
+        <v>29</v>
+      </c>
+      <c r="P9" s="4">
+        <v>47</v>
+      </c>
+      <c r="Q9" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="R9" t="s">
+        <v>31</v>
+      </c>
+      <c r="S9" t="s">
+        <v>24</v>
+      </c>
+      <c r="T9" t="s">
+        <v>24</v>
+      </c>
+      <c r="U9" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>56</v>
+      </c>
+      <c r="C10" t="s">
+        <v>62</v>
+      </c>
+      <c r="D10" t="s">
+        <v>23</v>
+      </c>
+      <c r="E10" t="s">
+        <v>24</v>
+      </c>
+      <c r="F10" t="s">
+        <v>24</v>
+      </c>
+      <c r="G10" t="s">
+        <v>63</v>
+      </c>
+      <c r="H10" t="s">
+        <v>24</v>
+      </c>
+      <c r="I10" t="s">
+        <v>24</v>
+      </c>
+      <c r="J10" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="K10" t="s">
+        <v>24</v>
+      </c>
+      <c r="L10" t="s">
+        <v>26</v>
+      </c>
+      <c r="M10" t="s">
+        <v>27</v>
+      </c>
+      <c r="N10" t="s">
+        <v>28</v>
+      </c>
+      <c r="O10" t="s">
+        <v>29</v>
+      </c>
+      <c r="P10" s="4">
+        <v>42</v>
+      </c>
+      <c r="Q10" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="R10" t="s">
+        <v>65</v>
+      </c>
+      <c r="S10" t="s">
+        <v>39</v>
+      </c>
+      <c r="T10" t="s">
+        <v>24</v>
+      </c>
+      <c r="U10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="11" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>66</v>
+      </c>
+      <c r="C11" t="s">
+        <v>67</v>
+      </c>
+      <c r="D11" t="s">
+        <v>68</v>
+      </c>
+      <c r="E11" t="s">
+        <v>24</v>
+      </c>
+      <c r="F11" t="s">
+        <v>24</v>
+      </c>
+      <c r="G11" t="s">
+        <v>24</v>
+      </c>
+      <c r="H11" t="s">
+        <v>24</v>
+      </c>
+      <c r="I11" t="s">
+        <v>24</v>
+      </c>
+      <c r="J11" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="K11" t="s">
+        <v>24</v>
+      </c>
+      <c r="L11" t="s">
+        <v>26</v>
+      </c>
+      <c r="M11" t="s">
+        <v>27</v>
+      </c>
+      <c r="N11" t="s">
+        <v>28</v>
+      </c>
+      <c r="O11" t="s">
+        <v>29</v>
+      </c>
+      <c r="P11" s="4">
+        <v>41</v>
+      </c>
+      <c r="Q11" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="R11" t="s">
+        <v>70</v>
+      </c>
+      <c r="S11" t="s">
+        <v>24</v>
+      </c>
+      <c r="T11" t="s">
+        <v>24</v>
+      </c>
+      <c r="U11" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="12" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
+        <v>71</v>
+      </c>
+      <c r="C12" t="s">
+        <v>72</v>
+      </c>
+      <c r="D12" t="s">
+        <v>73</v>
+      </c>
+      <c r="E12" t="s">
+        <v>24</v>
+      </c>
+      <c r="F12" t="s">
+        <v>24</v>
+      </c>
+      <c r="G12" t="s">
+        <v>24</v>
+      </c>
+      <c r="H12" t="s">
+        <v>24</v>
+      </c>
+      <c r="I12" t="s">
+        <v>24</v>
+      </c>
+      <c r="J12" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="K12" t="s">
+        <v>24</v>
+      </c>
+      <c r="L12" t="s">
+        <v>26</v>
+      </c>
+      <c r="M12" t="s">
+        <v>27</v>
+      </c>
+      <c r="N12" t="s">
+        <v>28</v>
+      </c>
+      <c r="O12" t="s">
+        <v>29</v>
+      </c>
+      <c r="P12" s="4">
+        <v>41</v>
+      </c>
+      <c r="Q12" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="R12" t="s">
+        <v>75</v>
+      </c>
+      <c r="S12" t="s">
+        <v>24</v>
+      </c>
+      <c r="T12" t="s">
+        <v>24</v>
+      </c>
+      <c r="U12" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="13" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>76</v>
+      </c>
+      <c r="C13" t="s">
+        <v>77</v>
+      </c>
+      <c r="D13" t="s">
+        <v>78</v>
+      </c>
+      <c r="E13" t="s">
+        <v>24</v>
+      </c>
+      <c r="F13" t="s">
+        <v>24</v>
+      </c>
+      <c r="G13" t="s">
+        <v>24</v>
+      </c>
+      <c r="H13" t="s">
+        <v>24</v>
+      </c>
+      <c r="I13" t="s">
+        <v>24</v>
+      </c>
+      <c r="J13" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="K13" t="s">
+        <v>24</v>
+      </c>
+      <c r="L13" t="s">
+        <v>26</v>
+      </c>
+      <c r="M13" t="s">
+        <v>27</v>
+      </c>
+      <c r="N13" t="s">
+        <v>28</v>
+      </c>
+      <c r="O13" t="s">
+        <v>29</v>
+      </c>
+      <c r="P13" s="4">
+        <v>41</v>
+      </c>
+      <c r="Q13" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="R13" t="s">
+        <v>80</v>
+      </c>
+      <c r="S13" t="s">
+        <v>24</v>
+      </c>
+      <c r="T13" t="s">
+        <v>24</v>
+      </c>
+      <c r="U13" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="14" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
+        <v>81</v>
+      </c>
+      <c r="C14" t="s">
+        <v>82</v>
+      </c>
+      <c r="D14" t="s">
+        <v>23</v>
+      </c>
+      <c r="E14" t="s">
+        <v>24</v>
+      </c>
+      <c r="F14" t="s">
+        <v>24</v>
+      </c>
+      <c r="G14" t="s">
+        <v>83</v>
+      </c>
+      <c r="H14" t="s">
+        <v>24</v>
+      </c>
+      <c r="I14" t="s">
+        <v>24</v>
+      </c>
+      <c r="J14" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="K14" t="s">
+        <v>24</v>
+      </c>
+      <c r="L14" t="s">
+        <v>26</v>
+      </c>
+      <c r="M14" t="s">
+        <v>27</v>
+      </c>
+      <c r="N14" t="s">
+        <v>28</v>
+      </c>
+      <c r="O14" t="s">
+        <v>29</v>
+      </c>
+      <c r="P14" s="4">
+        <v>39</v>
+      </c>
+      <c r="Q14" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="R14" t="s">
+        <v>85</v>
+      </c>
+      <c r="S14" t="s">
+        <v>24</v>
+      </c>
+      <c r="T14" t="s">
+        <v>24</v>
+      </c>
+      <c r="U14" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="15" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>33</v>
+      </c>
+      <c r="C15" t="s">
+        <v>86</v>
+      </c>
+      <c r="D15" t="s">
+        <v>87</v>
+      </c>
+      <c r="E15" t="s">
+        <v>24</v>
+      </c>
+      <c r="F15" t="s">
+        <v>24</v>
+      </c>
+      <c r="G15" t="s">
+        <v>88</v>
+      </c>
+      <c r="H15" t="s">
+        <v>24</v>
+      </c>
+      <c r="I15" t="s">
+        <v>24</v>
+      </c>
+      <c r="J15" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="K15" t="s">
+        <v>24</v>
+      </c>
+      <c r="L15" t="s">
+        <v>26</v>
+      </c>
+      <c r="M15" t="s">
+        <v>27</v>
+      </c>
+      <c r="N15" t="s">
+        <v>28</v>
+      </c>
+      <c r="O15" t="s">
+        <v>29</v>
+      </c>
+      <c r="P15" s="4">
+        <v>36</v>
+      </c>
+      <c r="Q15" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="R15" t="s">
+        <v>90</v>
+      </c>
+      <c r="S15" t="s">
+        <v>91</v>
+      </c>
+      <c r="T15" t="s">
+        <v>24</v>
+      </c>
+      <c r="U15" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="16" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="s">
+        <v>92</v>
+      </c>
+      <c r="C16" t="s">
+        <v>93</v>
+      </c>
+      <c r="D16" t="s">
+        <v>51</v>
+      </c>
+      <c r="E16" t="s">
+        <v>24</v>
+      </c>
+      <c r="F16" t="s">
+        <v>24</v>
+      </c>
+      <c r="G16" t="s">
+        <v>94</v>
+      </c>
+      <c r="H16" t="s">
+        <v>24</v>
+      </c>
+      <c r="I16" t="s">
+        <v>24</v>
+      </c>
+      <c r="J16" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="K16" t="s">
+        <v>24</v>
+      </c>
+      <c r="L16" t="s">
+        <v>26</v>
+      </c>
+      <c r="M16" t="s">
+        <v>27</v>
+      </c>
+      <c r="N16" t="s">
+        <v>28</v>
+      </c>
+      <c r="O16" t="s">
+        <v>29</v>
+      </c>
+      <c r="P16" s="4">
+        <v>36</v>
+      </c>
+      <c r="Q16" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="R16" t="s">
+        <v>96</v>
+      </c>
+      <c r="S16" t="s">
+        <v>97</v>
+      </c>
+      <c r="T16" t="s">
+        <v>24</v>
+      </c>
+      <c r="U16" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="17" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" t="s">
+        <v>98</v>
+      </c>
+      <c r="C17" t="s">
+        <v>99</v>
+      </c>
+      <c r="D17" t="s">
+        <v>51</v>
+      </c>
+      <c r="E17" t="s">
+        <v>24</v>
+      </c>
+      <c r="F17" t="s">
+        <v>24</v>
+      </c>
+      <c r="G17" t="s">
+        <v>97</v>
+      </c>
+      <c r="H17" t="s">
+        <v>24</v>
+      </c>
+      <c r="I17" t="s">
+        <v>24</v>
+      </c>
+      <c r="J17" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="K17" t="s">
+        <v>24</v>
+      </c>
+      <c r="L17" t="s">
+        <v>26</v>
+      </c>
+      <c r="M17" t="s">
+        <v>27</v>
+      </c>
+      <c r="N17" t="s">
+        <v>28</v>
+      </c>
+      <c r="O17" t="s">
+        <v>29</v>
+      </c>
+      <c r="P17" s="4">
+        <v>33</v>
+      </c>
+      <c r="Q17" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="R17" t="s">
+        <v>101</v>
+      </c>
+      <c r="S17" t="s">
+        <v>97</v>
+      </c>
+      <c r="T17" t="s">
+        <v>24</v>
+      </c>
+      <c r="U17" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="18" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" t="s">
+        <v>92</v>
+      </c>
+      <c r="C18" t="s">
+        <v>102</v>
+      </c>
+      <c r="D18" t="s">
+        <v>51</v>
+      </c>
+      <c r="E18" t="s">
+        <v>24</v>
+      </c>
+      <c r="F18" t="s">
+        <v>24</v>
+      </c>
+      <c r="G18" t="s">
+        <v>103</v>
+      </c>
+      <c r="H18" t="s">
+        <v>24</v>
+      </c>
+      <c r="I18" t="s">
+        <v>24</v>
+      </c>
+      <c r="J18" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="K18" t="s">
+        <v>24</v>
+      </c>
+      <c r="L18" t="s">
+        <v>26</v>
+      </c>
+      <c r="M18" t="s">
+        <v>27</v>
+      </c>
+      <c r="N18" t="s">
+        <v>28</v>
+      </c>
+      <c r="O18" t="s">
+        <v>29</v>
+      </c>
+      <c r="P18" s="4">
+        <v>33</v>
+      </c>
+      <c r="Q18" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="R18" t="s">
+        <v>101</v>
+      </c>
+      <c r="S18" t="s">
+        <v>103</v>
+      </c>
+      <c r="T18" t="s">
+        <v>24</v>
+      </c>
+      <c r="U18" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="19" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" t="s">
+        <v>105</v>
+      </c>
+      <c r="C19" t="s">
+        <v>106</v>
+      </c>
+      <c r="D19" t="s">
+        <v>58</v>
+      </c>
+      <c r="E19" t="s">
+        <v>24</v>
+      </c>
+      <c r="F19" t="s">
+        <v>24</v>
+      </c>
+      <c r="G19" t="s">
+        <v>107</v>
+      </c>
+      <c r="H19" t="s">
+        <v>24</v>
+      </c>
+      <c r="I19" t="s">
+        <v>24</v>
+      </c>
+      <c r="J19" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="K19" t="s">
+        <v>24</v>
+      </c>
+      <c r="L19" t="s">
+        <v>26</v>
+      </c>
+      <c r="M19" t="s">
+        <v>27</v>
+      </c>
+      <c r="N19" t="s">
+        <v>28</v>
+      </c>
+      <c r="O19" t="s">
+        <v>29</v>
+      </c>
+      <c r="P19" s="4">
+        <v>32</v>
+      </c>
+      <c r="Q19" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="R19" t="s">
+        <v>101</v>
+      </c>
+      <c r="S19" t="s">
+        <v>107</v>
+      </c>
+      <c r="T19" t="s">
+        <v>24</v>
+      </c>
+      <c r="U19" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="20" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" t="s">
+        <v>33</v>
+      </c>
+      <c r="C20" t="s">
+        <v>109</v>
+      </c>
+      <c r="D20" t="s">
+        <v>73</v>
+      </c>
+      <c r="E20" t="s">
+        <v>24</v>
+      </c>
+      <c r="F20" t="s">
+        <v>24</v>
+      </c>
+      <c r="G20" t="s">
+        <v>97</v>
+      </c>
+      <c r="H20" t="s">
+        <v>24</v>
+      </c>
+      <c r="I20" t="s">
+        <v>24</v>
+      </c>
+      <c r="J20" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="K20" t="s">
+        <v>24</v>
+      </c>
+      <c r="L20" t="s">
+        <v>26</v>
+      </c>
+      <c r="M20" t="s">
+        <v>27</v>
+      </c>
+      <c r="N20" t="s">
+        <v>28</v>
+      </c>
+      <c r="O20" t="s">
+        <v>29</v>
+      </c>
+      <c r="P20" s="4">
+        <v>29</v>
+      </c>
+      <c r="Q20" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="R20" t="s">
+        <v>111</v>
+      </c>
+      <c r="S20" t="s">
+        <v>97</v>
+      </c>
+      <c r="T20" t="s">
+        <v>24</v>
+      </c>
+      <c r="U20" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="21" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21" t="s">
+        <v>112</v>
+      </c>
+      <c r="C21" t="s">
+        <v>113</v>
+      </c>
+      <c r="D21" t="s">
+        <v>23</v>
+      </c>
+      <c r="E21" t="s">
+        <v>24</v>
+      </c>
+      <c r="F21" t="s">
+        <v>24</v>
+      </c>
+      <c r="G21" t="s">
+        <v>103</v>
+      </c>
+      <c r="H21" t="s">
+        <v>24</v>
+      </c>
+      <c r="I21" t="s">
+        <v>24</v>
+      </c>
+      <c r="J21" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="K21" t="s">
+        <v>24</v>
+      </c>
+      <c r="L21" t="s">
+        <v>26</v>
+      </c>
+      <c r="M21" t="s">
+        <v>27</v>
+      </c>
+      <c r="N21" t="s">
+        <v>28</v>
+      </c>
+      <c r="O21" t="s">
+        <v>29</v>
+      </c>
+      <c r="P21" s="4">
+        <v>28</v>
+      </c>
+      <c r="Q21" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="R21" t="s">
+        <v>101</v>
+      </c>
+      <c r="S21" t="s">
+        <v>103</v>
+      </c>
+      <c r="T21" t="s">
+        <v>24</v>
+      </c>
+      <c r="U21" t="s">
+        <v>32</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:T1"/>
+  <autoFilter ref="A1:U1"/>
+  <dataValidations count="2">
+    <dataValidation type="list" sqref="U10:U21">
+      <formula1>"A ENVOYER,Envoyee,En attente,Refusee,Entretien,Retiree"</formula1>
+    </dataValidation>
+    <dataValidation type="list" sqref="U2:U21">
+      <formula1>"A ENVOYER,Envoyee,En attente,Refusee,Entretien,Retiree"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="J2" r:id="rId1"/>
+    <hyperlink ref="J3" r:id="rId2"/>
+    <hyperlink ref="J4" r:id="rId3"/>
+    <hyperlink ref="J5" r:id="rId4"/>
+    <hyperlink ref="J6" r:id="rId5"/>
+    <hyperlink ref="J7" r:id="rId6"/>
+    <hyperlink ref="J8" r:id="rId7"/>
+    <hyperlink ref="J9" r:id="rId8"/>
+    <hyperlink ref="J10" r:id="rId9"/>
+    <hyperlink ref="J11" r:id="rId10"/>
+    <hyperlink ref="J12" r:id="rId11"/>
+    <hyperlink ref="J13" r:id="rId12"/>
+    <hyperlink ref="J14" r:id="rId13"/>
+    <hyperlink ref="J15" r:id="rId14"/>
+    <hyperlink ref="J16" r:id="rId15"/>
+    <hyperlink ref="J17" r:id="rId16"/>
+    <hyperlink ref="J18" r:id="rId17"/>
+    <hyperlink ref="J19" r:id="rId18"/>
+    <hyperlink ref="J20" r:id="rId19"/>
+    <hyperlink ref="J21" r:id="rId20"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -887,23 +2231,23 @@
   <sheetData>
     <row r="1" ht="25" customHeight="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>49</v>
+        <v>115</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>50</v>
+        <v>116</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>51</v>
+        <v>117</v>
       </c>
       <c r="B2">
-        <v>3</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>52</v>
+        <v>118</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -911,15 +2255,15 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>53</v>
+        <v>119</v>
       </c>
       <c r="B4">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>54</v>
+        <v>120</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -927,39 +2271,39 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>55</v>
+        <v>121</v>
       </c>
       <c r="B6">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>56</v>
+        <v>122</v>
       </c>
       <c r="B7">
-        <v>1</v>
+        <v>17</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>57</v>
+        <v>123</v>
       </c>
       <c r="B8">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>58</v>
+        <v>124</v>
       </c>
       <c r="B9">
-        <v>2</v>
+        <v>20</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>59</v>
+        <v>125</v>
       </c>
       <c r="B10" t="s">
         <v>28</v>

</xml_diff>